<commit_message>
Updating the model for Ulmeni
</commit_message>
<xml_diff>
--- a/Market Fundamentals/Transelectrica_data/Cons_Prod_final/Weekly_Consumption_2026.xlsx
+++ b/Market Fundamentals/Transelectrica_data/Cons_Prod_final/Weekly_Consumption_2026.xlsx
@@ -8188,7 +8188,7 @@
         <v>1</v>
       </c>
       <c r="C290">
-        <v>5020</v>
+        <v>5030</v>
       </c>
       <c r="D290" t="s">
         <v>292</v>
@@ -8216,7 +8216,7 @@
         <v>3</v>
       </c>
       <c r="C292">
-        <v>4950</v>
+        <v>4920</v>
       </c>
       <c r="D292" t="s">
         <v>294</v>
@@ -8230,7 +8230,7 @@
         <v>4</v>
       </c>
       <c r="C293">
-        <v>4890</v>
+        <v>4870</v>
       </c>
       <c r="D293" t="s">
         <v>295</v>
@@ -8244,7 +8244,7 @@
         <v>5</v>
       </c>
       <c r="C294">
-        <v>4830</v>
+        <v>4820</v>
       </c>
       <c r="D294" t="s">
         <v>296</v>
@@ -8258,7 +8258,7 @@
         <v>6</v>
       </c>
       <c r="C295">
-        <v>4780</v>
+        <v>4770</v>
       </c>
       <c r="D295" t="s">
         <v>297</v>
@@ -8272,7 +8272,7 @@
         <v>7</v>
       </c>
       <c r="C296">
-        <v>4740</v>
+        <v>4720</v>
       </c>
       <c r="D296" t="s">
         <v>298</v>
@@ -8286,7 +8286,7 @@
         <v>8</v>
       </c>
       <c r="C297">
-        <v>4710</v>
+        <v>4690</v>
       </c>
       <c r="D297" t="s">
         <v>299</v>
@@ -8300,7 +8300,7 @@
         <v>9</v>
       </c>
       <c r="C298">
-        <v>4680</v>
+        <v>4640</v>
       </c>
       <c r="D298" t="s">
         <v>300</v>
@@ -8314,7 +8314,7 @@
         <v>10</v>
       </c>
       <c r="C299">
-        <v>4670</v>
+        <v>4610</v>
       </c>
       <c r="D299" t="s">
         <v>301</v>
@@ -8328,7 +8328,7 @@
         <v>11</v>
       </c>
       <c r="C300">
-        <v>4660</v>
+        <v>4590</v>
       </c>
       <c r="D300" t="s">
         <v>302</v>
@@ -8342,7 +8342,7 @@
         <v>12</v>
       </c>
       <c r="C301">
-        <v>4650</v>
+        <v>4560</v>
       </c>
       <c r="D301" t="s">
         <v>303</v>
@@ -8356,7 +8356,7 @@
         <v>13</v>
       </c>
       <c r="C302">
-        <v>4650</v>
+        <v>4540</v>
       </c>
       <c r="D302" t="s">
         <v>304</v>
@@ -8370,7 +8370,7 @@
         <v>14</v>
       </c>
       <c r="C303">
-        <v>4650</v>
+        <v>4530</v>
       </c>
       <c r="D303" t="s">
         <v>305</v>
@@ -8384,7 +8384,7 @@
         <v>15</v>
       </c>
       <c r="C304">
-        <v>4660</v>
+        <v>4530</v>
       </c>
       <c r="D304" t="s">
         <v>306</v>
@@ -8398,7 +8398,7 @@
         <v>16</v>
       </c>
       <c r="C305">
-        <v>4670</v>
+        <v>4520</v>
       </c>
       <c r="D305" t="s">
         <v>307</v>
@@ -8412,7 +8412,7 @@
         <v>17</v>
       </c>
       <c r="C306">
-        <v>4690</v>
+        <v>4500</v>
       </c>
       <c r="D306" t="s">
         <v>308</v>
@@ -8426,7 +8426,7 @@
         <v>18</v>
       </c>
       <c r="C307">
-        <v>4700</v>
+        <v>4490</v>
       </c>
       <c r="D307" t="s">
         <v>309</v>
@@ -8440,7 +8440,7 @@
         <v>19</v>
       </c>
       <c r="C308">
-        <v>4700</v>
+        <v>4500</v>
       </c>
       <c r="D308" t="s">
         <v>310</v>
@@ -8454,7 +8454,7 @@
         <v>20</v>
       </c>
       <c r="C309">
-        <v>4710</v>
+        <v>4510</v>
       </c>
       <c r="D309" t="s">
         <v>311</v>
@@ -8468,7 +8468,7 @@
         <v>21</v>
       </c>
       <c r="C310">
-        <v>4710</v>
+        <v>4550</v>
       </c>
       <c r="D310" t="s">
         <v>312</v>
@@ -8482,7 +8482,7 @@
         <v>22</v>
       </c>
       <c r="C311">
-        <v>4710</v>
+        <v>4570</v>
       </c>
       <c r="D311" t="s">
         <v>313</v>
@@ -8496,7 +8496,7 @@
         <v>23</v>
       </c>
       <c r="C312">
-        <v>4710</v>
+        <v>4590</v>
       </c>
       <c r="D312" t="s">
         <v>314</v>
@@ -8510,7 +8510,7 @@
         <v>24</v>
       </c>
       <c r="C313">
-        <v>4710</v>
+        <v>4610</v>
       </c>
       <c r="D313" t="s">
         <v>315</v>
@@ -8524,7 +8524,7 @@
         <v>25</v>
       </c>
       <c r="C314">
-        <v>4720</v>
+        <v>4650</v>
       </c>
       <c r="D314" t="s">
         <v>316</v>
@@ -8538,7 +8538,7 @@
         <v>26</v>
       </c>
       <c r="C315">
-        <v>4730</v>
+        <v>4670</v>
       </c>
       <c r="D315" t="s">
         <v>317</v>
@@ -8552,7 +8552,7 @@
         <v>27</v>
       </c>
       <c r="C316">
-        <v>4750</v>
+        <v>4690</v>
       </c>
       <c r="D316" t="s">
         <v>318</v>
@@ -8566,7 +8566,7 @@
         <v>28</v>
       </c>
       <c r="C317">
-        <v>4780</v>
+        <v>4710</v>
       </c>
       <c r="D317" t="s">
         <v>319</v>
@@ -8580,7 +8580,7 @@
         <v>29</v>
       </c>
       <c r="C318">
-        <v>4800</v>
+        <v>4740</v>
       </c>
       <c r="D318" t="s">
         <v>320</v>
@@ -8594,7 +8594,7 @@
         <v>30</v>
       </c>
       <c r="C319">
-        <v>4830</v>
+        <v>4760</v>
       </c>
       <c r="D319" t="s">
         <v>321</v>
@@ -8608,7 +8608,7 @@
         <v>31</v>
       </c>
       <c r="C320">
-        <v>4840</v>
+        <v>4760</v>
       </c>
       <c r="D320" t="s">
         <v>322</v>
@@ -8622,7 +8622,7 @@
         <v>32</v>
       </c>
       <c r="C321">
-        <v>4850</v>
+        <v>4740</v>
       </c>
       <c r="D321" t="s">
         <v>323</v>
@@ -8636,7 +8636,7 @@
         <v>33</v>
       </c>
       <c r="C322">
-        <v>4850</v>
+        <v>4720</v>
       </c>
       <c r="D322" t="s">
         <v>324</v>
@@ -8650,7 +8650,7 @@
         <v>34</v>
       </c>
       <c r="C323">
-        <v>4800</v>
+        <v>4690</v>
       </c>
       <c r="D323" t="s">
         <v>325</v>
@@ -8664,7 +8664,7 @@
         <v>35</v>
       </c>
       <c r="C324">
-        <v>4740</v>
+        <v>4640</v>
       </c>
       <c r="D324" t="s">
         <v>326</v>
@@ -8678,7 +8678,7 @@
         <v>36</v>
       </c>
       <c r="C325">
-        <v>4650</v>
+        <v>4550</v>
       </c>
       <c r="D325" t="s">
         <v>327</v>
@@ -8692,7 +8692,7 @@
         <v>37</v>
       </c>
       <c r="C326">
-        <v>4540</v>
+        <v>4370</v>
       </c>
       <c r="D326" t="s">
         <v>328</v>
@@ -8706,7 +8706,7 @@
         <v>38</v>
       </c>
       <c r="C327">
-        <v>4400</v>
+        <v>4210</v>
       </c>
       <c r="D327" t="s">
         <v>329</v>
@@ -8720,7 +8720,7 @@
         <v>39</v>
       </c>
       <c r="C328">
-        <v>4250</v>
+        <v>4060</v>
       </c>
       <c r="D328" t="s">
         <v>330</v>
@@ -8734,7 +8734,7 @@
         <v>40</v>
       </c>
       <c r="C329">
-        <v>4090</v>
+        <v>3920</v>
       </c>
       <c r="D329" t="s">
         <v>331</v>
@@ -8748,7 +8748,7 @@
         <v>41</v>
       </c>
       <c r="C330">
-        <v>3920</v>
+        <v>3790</v>
       </c>
       <c r="D330" t="s">
         <v>332</v>
@@ -8762,7 +8762,7 @@
         <v>42</v>
       </c>
       <c r="C331">
-        <v>3770</v>
+        <v>3660</v>
       </c>
       <c r="D331" t="s">
         <v>333</v>
@@ -8776,7 +8776,7 @@
         <v>43</v>
       </c>
       <c r="C332">
-        <v>3620</v>
+        <v>3500</v>
       </c>
       <c r="D332" t="s">
         <v>334</v>
@@ -8790,7 +8790,7 @@
         <v>44</v>
       </c>
       <c r="C333">
-        <v>3490</v>
+        <v>3370</v>
       </c>
       <c r="D333" t="s">
         <v>335</v>
@@ -8804,7 +8804,7 @@
         <v>45</v>
       </c>
       <c r="C334">
-        <v>3380</v>
+        <v>3220</v>
       </c>
       <c r="D334" t="s">
         <v>336</v>
@@ -8818,7 +8818,7 @@
         <v>46</v>
       </c>
       <c r="C335">
-        <v>3300</v>
+        <v>3110</v>
       </c>
       <c r="D335" t="s">
         <v>337</v>
@@ -8832,7 +8832,7 @@
         <v>47</v>
       </c>
       <c r="C336">
-        <v>3230</v>
+        <v>3050</v>
       </c>
       <c r="D336" t="s">
         <v>338</v>
@@ -8846,7 +8846,7 @@
         <v>48</v>
       </c>
       <c r="C337">
-        <v>3190</v>
+        <v>3020</v>
       </c>
       <c r="D337" t="s">
         <v>339</v>
@@ -8860,7 +8860,7 @@
         <v>49</v>
       </c>
       <c r="C338">
-        <v>3160</v>
+        <v>3000</v>
       </c>
       <c r="D338" t="s">
         <v>340</v>
@@ -8874,7 +8874,7 @@
         <v>50</v>
       </c>
       <c r="C339">
-        <v>3150</v>
+        <v>2990</v>
       </c>
       <c r="D339" t="s">
         <v>341</v>
@@ -8888,7 +8888,7 @@
         <v>51</v>
       </c>
       <c r="C340">
-        <v>3150</v>
+        <v>2990</v>
       </c>
       <c r="D340" t="s">
         <v>342</v>
@@ -8902,7 +8902,7 @@
         <v>52</v>
       </c>
       <c r="C341">
-        <v>3150</v>
+        <v>3020</v>
       </c>
       <c r="D341" t="s">
         <v>343</v>
@@ -8916,7 +8916,7 @@
         <v>53</v>
       </c>
       <c r="C342">
-        <v>3170</v>
+        <v>3050</v>
       </c>
       <c r="D342" t="s">
         <v>344</v>
@@ -8930,7 +8930,7 @@
         <v>54</v>
       </c>
       <c r="C343">
-        <v>3190</v>
+        <v>3080</v>
       </c>
       <c r="D343" t="s">
         <v>345</v>
@@ -8944,7 +8944,7 @@
         <v>55</v>
       </c>
       <c r="C344">
-        <v>3210</v>
+        <v>3110</v>
       </c>
       <c r="D344" t="s">
         <v>346</v>
@@ -8958,7 +8958,7 @@
         <v>56</v>
       </c>
       <c r="C345">
-        <v>3240</v>
+        <v>3160</v>
       </c>
       <c r="D345" t="s">
         <v>347</v>
@@ -8972,7 +8972,7 @@
         <v>57</v>
       </c>
       <c r="C346">
-        <v>3270</v>
+        <v>3210</v>
       </c>
       <c r="D346" t="s">
         <v>348</v>
@@ -8986,7 +8986,7 @@
         <v>58</v>
       </c>
       <c r="C347">
-        <v>3310</v>
+        <v>3270</v>
       </c>
       <c r="D347" t="s">
         <v>349</v>
@@ -9000,7 +9000,7 @@
         <v>59</v>
       </c>
       <c r="C348">
-        <v>3350</v>
+        <v>3330</v>
       </c>
       <c r="D348" t="s">
         <v>350</v>
@@ -9014,7 +9014,7 @@
         <v>60</v>
       </c>
       <c r="C349">
-        <v>3400</v>
+        <v>3390</v>
       </c>
       <c r="D349" t="s">
         <v>351</v>
@@ -9056,7 +9056,7 @@
         <v>63</v>
       </c>
       <c r="C352">
-        <v>3590</v>
+        <v>3580</v>
       </c>
       <c r="D352" t="s">
         <v>354</v>
@@ -9070,7 +9070,7 @@
         <v>64</v>
       </c>
       <c r="C353">
-        <v>3680</v>
+        <v>3660</v>
       </c>
       <c r="D353" t="s">
         <v>355</v>
@@ -9084,7 +9084,7 @@
         <v>65</v>
       </c>
       <c r="C354">
-        <v>3780</v>
+        <v>3750</v>
       </c>
       <c r="D354" t="s">
         <v>356</v>
@@ -9098,7 +9098,7 @@
         <v>66</v>
       </c>
       <c r="C355">
-        <v>3910</v>
+        <v>3870</v>
       </c>
       <c r="D355" t="s">
         <v>357</v>
@@ -9112,7 +9112,7 @@
         <v>67</v>
       </c>
       <c r="C356">
-        <v>4050</v>
+        <v>4010</v>
       </c>
       <c r="D356" t="s">
         <v>358</v>
@@ -9126,7 +9126,7 @@
         <v>68</v>
       </c>
       <c r="C357">
-        <v>4210</v>
+        <v>4170</v>
       </c>
       <c r="D357" t="s">
         <v>359</v>
@@ -9182,7 +9182,7 @@
         <v>72</v>
       </c>
       <c r="C361">
-        <v>4910</v>
+        <v>4920</v>
       </c>
       <c r="D361" t="s">
         <v>363</v>
@@ -9196,7 +9196,7 @@
         <v>73</v>
       </c>
       <c r="C362">
-        <v>5070</v>
+        <v>5090</v>
       </c>
       <c r="D362" t="s">
         <v>364</v>
@@ -9238,7 +9238,7 @@
         <v>76</v>
       </c>
       <c r="C365">
-        <v>5520</v>
+        <v>5510</v>
       </c>
       <c r="D365" t="s">
         <v>367</v>
@@ -9252,7 +9252,7 @@
         <v>77</v>
       </c>
       <c r="C366">
-        <v>5650</v>
+        <v>5670</v>
       </c>
       <c r="D366" t="s">
         <v>368</v>
@@ -9266,7 +9266,7 @@
         <v>78</v>
       </c>
       <c r="C367">
-        <v>5780</v>
+        <v>5810</v>
       </c>
       <c r="D367" t="s">
         <v>369</v>
@@ -9280,7 +9280,7 @@
         <v>79</v>
       </c>
       <c r="C368">
-        <v>5900</v>
+        <v>5920</v>
       </c>
       <c r="D368" t="s">
         <v>370</v>
@@ -9294,7 +9294,7 @@
         <v>80</v>
       </c>
       <c r="C369">
-        <v>5980</v>
+        <v>6000</v>
       </c>
       <c r="D369" t="s">
         <v>371</v>
@@ -9308,7 +9308,7 @@
         <v>81</v>
       </c>
       <c r="C370">
-        <v>6030</v>
+        <v>6050</v>
       </c>
       <c r="D370" t="s">
         <v>372</v>
@@ -9322,7 +9322,7 @@
         <v>82</v>
       </c>
       <c r="C371">
-        <v>6050</v>
+        <v>6070</v>
       </c>
       <c r="D371" t="s">
         <v>373</v>
@@ -9336,7 +9336,7 @@
         <v>83</v>
       </c>
       <c r="C372">
-        <v>6050</v>
+        <v>6060</v>
       </c>
       <c r="D372" t="s">
         <v>374</v>
@@ -9350,7 +9350,7 @@
         <v>84</v>
       </c>
       <c r="C373">
-        <v>6000</v>
+        <v>6020</v>
       </c>
       <c r="D373" t="s">
         <v>375</v>
@@ -9364,7 +9364,7 @@
         <v>85</v>
       </c>
       <c r="C374">
-        <v>5850</v>
+        <v>5900</v>
       </c>
       <c r="D374" t="s">
         <v>376</v>
@@ -9378,7 +9378,7 @@
         <v>86</v>
       </c>
       <c r="C375">
-        <v>5700</v>
+        <v>5750</v>
       </c>
       <c r="D375" t="s">
         <v>377</v>
@@ -9392,7 +9392,7 @@
         <v>87</v>
       </c>
       <c r="C376">
-        <v>5580</v>
+        <v>5620</v>
       </c>
       <c r="D376" t="s">
         <v>378</v>
@@ -9406,7 +9406,7 @@
         <v>88</v>
       </c>
       <c r="C377">
-        <v>5540</v>
+        <v>5530</v>
       </c>
       <c r="D377" t="s">
         <v>379</v>
@@ -9420,7 +9420,7 @@
         <v>89</v>
       </c>
       <c r="C378">
-        <v>5430</v>
+        <v>5420</v>
       </c>
       <c r="D378" t="s">
         <v>380</v>
@@ -9434,7 +9434,7 @@
         <v>90</v>
       </c>
       <c r="C379">
-        <v>5320</v>
+        <v>5340</v>
       </c>
       <c r="D379" t="s">
         <v>381</v>
@@ -9448,7 +9448,7 @@
         <v>91</v>
       </c>
       <c r="C380">
-        <v>5150</v>
+        <v>5260</v>
       </c>
       <c r="D380" t="s">
         <v>382</v>
@@ -9462,7 +9462,7 @@
         <v>92</v>
       </c>
       <c r="C381">
-        <v>5080</v>
+        <v>5180</v>
       </c>
       <c r="D381" t="s">
         <v>383</v>
@@ -9476,7 +9476,7 @@
         <v>93</v>
       </c>
       <c r="C382">
-        <v>5020</v>
+        <v>5090</v>
       </c>
       <c r="D382" t="s">
         <v>384</v>
@@ -9490,7 +9490,7 @@
         <v>94</v>
       </c>
       <c r="C383">
-        <v>4980</v>
+        <v>5010</v>
       </c>
       <c r="D383" t="s">
         <v>385</v>
@@ -9504,7 +9504,7 @@
         <v>95</v>
       </c>
       <c r="C384">
-        <v>4950</v>
+        <v>4960</v>
       </c>
       <c r="D384" t="s">
         <v>386</v>
@@ -9518,7 +9518,7 @@
         <v>96</v>
       </c>
       <c r="C385">
-        <v>4930</v>
+        <v>4940</v>
       </c>
       <c r="D385" t="s">
         <v>387</v>
@@ -9532,7 +9532,7 @@
         <v>1</v>
       </c>
       <c r="C386">
-        <v>4940</v>
+        <v>4920</v>
       </c>
       <c r="D386" t="s">
         <v>388</v>

</xml_diff>

<commit_message>
Updating the model for Horeco
</commit_message>
<xml_diff>
--- a/Market Fundamentals/Transelectrica_data/Cons_Prod_final/Weekly_Consumption_2026.xlsx
+++ b/Market Fundamentals/Transelectrica_data/Cons_Prod_final/Weekly_Consumption_2026.xlsx
@@ -13852,7 +13852,7 @@
         <v>1</v>
       </c>
       <c r="C674">
-        <v>5440</v>
+        <v>5220</v>
       </c>
       <c r="D674" t="s">
         <v>676</v>
@@ -13866,7 +13866,7 @@
         <v>2</v>
       </c>
       <c r="C675">
-        <v>5400</v>
+        <v>5170</v>
       </c>
       <c r="D675" t="s">
         <v>677</v>
@@ -13880,7 +13880,7 @@
         <v>3</v>
       </c>
       <c r="C676">
-        <v>5350</v>
+        <v>5130</v>
       </c>
       <c r="D676" t="s">
         <v>678</v>
@@ -13894,7 +13894,7 @@
         <v>4</v>
       </c>
       <c r="C677">
-        <v>5260</v>
+        <v>5120</v>
       </c>
       <c r="D677" t="s">
         <v>679</v>
@@ -13908,7 +13908,7 @@
         <v>5</v>
       </c>
       <c r="C678">
-        <v>5180</v>
+        <v>5100</v>
       </c>
       <c r="D678" t="s">
         <v>680</v>
@@ -13922,7 +13922,7 @@
         <v>6</v>
       </c>
       <c r="C679">
-        <v>5130</v>
+        <v>5100</v>
       </c>
       <c r="D679" t="s">
         <v>681</v>
@@ -13950,7 +13950,7 @@
         <v>8</v>
       </c>
       <c r="C681">
-        <v>5090</v>
+        <v>5100</v>
       </c>
       <c r="D681" t="s">
         <v>683</v>
@@ -14006,7 +14006,7 @@
         <v>12</v>
       </c>
       <c r="C685">
-        <v>5100</v>
+        <v>5110</v>
       </c>
       <c r="D685" t="s">
         <v>687</v>
@@ -14020,7 +14020,7 @@
         <v>13</v>
       </c>
       <c r="C686">
-        <v>5110</v>
+        <v>5120</v>
       </c>
       <c r="D686" t="s">
         <v>688</v>
@@ -14034,7 +14034,7 @@
         <v>14</v>
       </c>
       <c r="C687">
-        <v>5110</v>
+        <v>5150</v>
       </c>
       <c r="D687" t="s">
         <v>689</v>
@@ -14048,7 +14048,7 @@
         <v>15</v>
       </c>
       <c r="C688">
-        <v>5120</v>
+        <v>5150</v>
       </c>
       <c r="D688" t="s">
         <v>690</v>
@@ -14062,7 +14062,7 @@
         <v>16</v>
       </c>
       <c r="C689">
-        <v>5130</v>
+        <v>5150</v>
       </c>
       <c r="D689" t="s">
         <v>691</v>
@@ -14076,7 +14076,7 @@
         <v>17</v>
       </c>
       <c r="C690">
-        <v>5140</v>
+        <v>5150</v>
       </c>
       <c r="D690" t="s">
         <v>692</v>
@@ -14104,7 +14104,7 @@
         <v>19</v>
       </c>
       <c r="C692">
-        <v>5170</v>
+        <v>5150</v>
       </c>
       <c r="D692" t="s">
         <v>694</v>
@@ -14118,7 +14118,7 @@
         <v>20</v>
       </c>
       <c r="C693">
-        <v>5190</v>
+        <v>5150</v>
       </c>
       <c r="D693" t="s">
         <v>695</v>
@@ -14132,7 +14132,7 @@
         <v>21</v>
       </c>
       <c r="C694">
-        <v>5220</v>
+        <v>5140</v>
       </c>
       <c r="D694" t="s">
         <v>696</v>
@@ -14146,7 +14146,7 @@
         <v>22</v>
       </c>
       <c r="C695">
-        <v>5270</v>
+        <v>5140</v>
       </c>
       <c r="D695" t="s">
         <v>697</v>
@@ -14160,7 +14160,7 @@
         <v>23</v>
       </c>
       <c r="C696">
-        <v>5340</v>
+        <v>5150</v>
       </c>
       <c r="D696" t="s">
         <v>698</v>
@@ -14174,7 +14174,7 @@
         <v>24</v>
       </c>
       <c r="C697">
-        <v>5430</v>
+        <v>5150</v>
       </c>
       <c r="D697" t="s">
         <v>699</v>
@@ -14188,7 +14188,7 @@
         <v>25</v>
       </c>
       <c r="C698">
-        <v>5540</v>
+        <v>5490</v>
       </c>
       <c r="D698" t="s">
         <v>700</v>
@@ -14202,7 +14202,7 @@
         <v>26</v>
       </c>
       <c r="C699">
-        <v>5680</v>
+        <v>5690</v>
       </c>
       <c r="D699" t="s">
         <v>701</v>
@@ -14230,7 +14230,7 @@
         <v>28</v>
       </c>
       <c r="C701">
-        <v>5990</v>
+        <v>6000</v>
       </c>
       <c r="D701" t="s">
         <v>703</v>
@@ -14244,7 +14244,7 @@
         <v>29</v>
       </c>
       <c r="C702">
-        <v>6150</v>
+        <v>6160</v>
       </c>
       <c r="D702" t="s">
         <v>704</v>
@@ -14272,7 +14272,7 @@
         <v>31</v>
       </c>
       <c r="C704">
-        <v>6410</v>
+        <v>6390</v>
       </c>
       <c r="D704" t="s">
         <v>706</v>
@@ -14286,7 +14286,7 @@
         <v>32</v>
       </c>
       <c r="C705">
-        <v>6500</v>
+        <v>6440</v>
       </c>
       <c r="D705" t="s">
         <v>707</v>
@@ -14300,7 +14300,7 @@
         <v>33</v>
       </c>
       <c r="C706">
-        <v>6550</v>
+        <v>6450</v>
       </c>
       <c r="D706" t="s">
         <v>708</v>
@@ -14314,7 +14314,7 @@
         <v>34</v>
       </c>
       <c r="C707">
-        <v>6540</v>
+        <v>6440</v>
       </c>
       <c r="D707" t="s">
         <v>709</v>
@@ -14328,7 +14328,7 @@
         <v>35</v>
       </c>
       <c r="C708">
-        <v>6500</v>
+        <v>6400</v>
       </c>
       <c r="D708" t="s">
         <v>710</v>
@@ -14342,7 +14342,7 @@
         <v>36</v>
       </c>
       <c r="C709">
-        <v>6410</v>
+        <v>6340</v>
       </c>
       <c r="D709" t="s">
         <v>711</v>
@@ -14356,7 +14356,7 @@
         <v>37</v>
       </c>
       <c r="C710">
-        <v>6290</v>
+        <v>6230</v>
       </c>
       <c r="D710" t="s">
         <v>712</v>
@@ -14370,7 +14370,7 @@
         <v>38</v>
       </c>
       <c r="C711">
-        <v>6140</v>
+        <v>6100</v>
       </c>
       <c r="D711" t="s">
         <v>713</v>
@@ -14384,7 +14384,7 @@
         <v>39</v>
       </c>
       <c r="C712">
-        <v>5970</v>
+        <v>5930</v>
       </c>
       <c r="D712" t="s">
         <v>714</v>
@@ -14398,7 +14398,7 @@
         <v>40</v>
       </c>
       <c r="C713">
-        <v>5800</v>
+        <v>5730</v>
       </c>
       <c r="D713" t="s">
         <v>715</v>
@@ -14412,7 +14412,7 @@
         <v>41</v>
       </c>
       <c r="C714">
-        <v>5620</v>
+        <v>5470</v>
       </c>
       <c r="D714" t="s">
         <v>716</v>
@@ -14426,7 +14426,7 @@
         <v>42</v>
       </c>
       <c r="C715">
-        <v>5450</v>
+        <v>5260</v>
       </c>
       <c r="D715" t="s">
         <v>717</v>
@@ -14440,7 +14440,7 @@
         <v>43</v>
       </c>
       <c r="C716">
-        <v>5290</v>
+        <v>5070</v>
       </c>
       <c r="D716" t="s">
         <v>718</v>
@@ -14454,7 +14454,7 @@
         <v>44</v>
       </c>
       <c r="C717">
-        <v>5150</v>
+        <v>4890</v>
       </c>
       <c r="D717" t="s">
         <v>719</v>
@@ -14468,7 +14468,7 @@
         <v>45</v>
       </c>
       <c r="C718">
-        <v>5030</v>
+        <v>4750</v>
       </c>
       <c r="D718" t="s">
         <v>720</v>
@@ -14482,7 +14482,7 @@
         <v>46</v>
       </c>
       <c r="C719">
-        <v>4920</v>
+        <v>4640</v>
       </c>
       <c r="D719" t="s">
         <v>721</v>
@@ -14496,7 +14496,7 @@
         <v>47</v>
       </c>
       <c r="C720">
-        <v>4820</v>
+        <v>4540</v>
       </c>
       <c r="D720" t="s">
         <v>722</v>
@@ -14510,7 +14510,7 @@
         <v>48</v>
       </c>
       <c r="C721">
-        <v>4740</v>
+        <v>4470</v>
       </c>
       <c r="D721" t="s">
         <v>723</v>
@@ -14524,7 +14524,7 @@
         <v>49</v>
       </c>
       <c r="C722">
-        <v>4680</v>
+        <v>4430</v>
       </c>
       <c r="D722" t="s">
         <v>724</v>
@@ -14538,7 +14538,7 @@
         <v>50</v>
       </c>
       <c r="C723">
-        <v>4630</v>
+        <v>4420</v>
       </c>
       <c r="D723" t="s">
         <v>725</v>
@@ -14552,7 +14552,7 @@
         <v>51</v>
       </c>
       <c r="C724">
-        <v>4600</v>
+        <v>4420</v>
       </c>
       <c r="D724" t="s">
         <v>726</v>
@@ -14566,7 +14566,7 @@
         <v>52</v>
       </c>
       <c r="C725">
-        <v>4580</v>
+        <v>4420</v>
       </c>
       <c r="D725" t="s">
         <v>727</v>
@@ -14580,7 +14580,7 @@
         <v>53</v>
       </c>
       <c r="C726">
-        <v>4580</v>
+        <v>4500</v>
       </c>
       <c r="D726" t="s">
         <v>728</v>
@@ -14594,7 +14594,7 @@
         <v>54</v>
       </c>
       <c r="C727">
-        <v>4590</v>
+        <v>4520</v>
       </c>
       <c r="D727" t="s">
         <v>729</v>
@@ -14608,7 +14608,7 @@
         <v>55</v>
       </c>
       <c r="C728">
-        <v>4610</v>
+        <v>4530</v>
       </c>
       <c r="D728" t="s">
         <v>730</v>
@@ -14622,7 +14622,7 @@
         <v>56</v>
       </c>
       <c r="C729">
-        <v>4640</v>
+        <v>4540</v>
       </c>
       <c r="D729" t="s">
         <v>731</v>
@@ -14636,7 +14636,7 @@
         <v>57</v>
       </c>
       <c r="C730">
-        <v>4670</v>
+        <v>4550</v>
       </c>
       <c r="D730" t="s">
         <v>732</v>
@@ -14650,7 +14650,7 @@
         <v>58</v>
       </c>
       <c r="C731">
-        <v>4710</v>
+        <v>4550</v>
       </c>
       <c r="D731" t="s">
         <v>733</v>
@@ -14664,7 +14664,7 @@
         <v>59</v>
       </c>
       <c r="C732">
-        <v>4740</v>
+        <v>4550</v>
       </c>
       <c r="D732" t="s">
         <v>734</v>
@@ -14678,7 +14678,7 @@
         <v>60</v>
       </c>
       <c r="C733">
-        <v>4780</v>
+        <v>4570</v>
       </c>
       <c r="D733" t="s">
         <v>735</v>
@@ -14692,7 +14692,7 @@
         <v>61</v>
       </c>
       <c r="C734">
-        <v>4820</v>
+        <v>4630</v>
       </c>
       <c r="D734" t="s">
         <v>736</v>
@@ -14706,7 +14706,7 @@
         <v>62</v>
       </c>
       <c r="C735">
-        <v>4870</v>
+        <v>4710</v>
       </c>
       <c r="D735" t="s">
         <v>737</v>
@@ -14720,7 +14720,7 @@
         <v>63</v>
       </c>
       <c r="C736">
-        <v>4930</v>
+        <v>4780</v>
       </c>
       <c r="D736" t="s">
         <v>738</v>
@@ -14734,7 +14734,7 @@
         <v>64</v>
       </c>
       <c r="C737">
-        <v>5000</v>
+        <v>4880</v>
       </c>
       <c r="D737" t="s">
         <v>739</v>
@@ -14748,7 +14748,7 @@
         <v>65</v>
       </c>
       <c r="C738">
-        <v>5100</v>
+        <v>4990</v>
       </c>
       <c r="D738" t="s">
         <v>740</v>
@@ -14762,7 +14762,7 @@
         <v>66</v>
       </c>
       <c r="C739">
-        <v>5210</v>
+        <v>5120</v>
       </c>
       <c r="D739" t="s">
         <v>741</v>
@@ -14776,7 +14776,7 @@
         <v>67</v>
       </c>
       <c r="C740">
-        <v>5340</v>
+        <v>5270</v>
       </c>
       <c r="D740" t="s">
         <v>742</v>
@@ -14790,7 +14790,7 @@
         <v>68</v>
       </c>
       <c r="C741">
-        <v>5480</v>
+        <v>5430</v>
       </c>
       <c r="D741" t="s">
         <v>743</v>
@@ -14804,7 +14804,7 @@
         <v>69</v>
       </c>
       <c r="C742">
-        <v>5630</v>
+        <v>5610</v>
       </c>
       <c r="D742" t="s">
         <v>744</v>
@@ -14832,7 +14832,7 @@
         <v>71</v>
       </c>
       <c r="C744">
-        <v>5940</v>
+        <v>5930</v>
       </c>
       <c r="D744" t="s">
         <v>746</v>
@@ -14846,7 +14846,7 @@
         <v>72</v>
       </c>
       <c r="C745">
-        <v>6090</v>
+        <v>6080</v>
       </c>
       <c r="D745" t="s">
         <v>747</v>
@@ -14860,7 +14860,7 @@
         <v>73</v>
       </c>
       <c r="C746">
-        <v>6250</v>
+        <v>6240</v>
       </c>
       <c r="D746" t="s">
         <v>748</v>
@@ -14874,7 +14874,7 @@
         <v>74</v>
       </c>
       <c r="C747">
-        <v>6410</v>
+        <v>6380</v>
       </c>
       <c r="D747" t="s">
         <v>749</v>
@@ -14888,7 +14888,7 @@
         <v>75</v>
       </c>
       <c r="C748">
-        <v>6580</v>
+        <v>6520</v>
       </c>
       <c r="D748" t="s">
         <v>750</v>
@@ -14902,7 +14902,7 @@
         <v>76</v>
       </c>
       <c r="C749">
-        <v>6740</v>
+        <v>6660</v>
       </c>
       <c r="D749" t="s">
         <v>751</v>
@@ -14916,7 +14916,7 @@
         <v>77</v>
       </c>
       <c r="C750">
-        <v>6890</v>
+        <v>6820</v>
       </c>
       <c r="D750" t="s">
         <v>752</v>
@@ -14930,7 +14930,7 @@
         <v>78</v>
       </c>
       <c r="C751">
-        <v>7020</v>
+        <v>6930</v>
       </c>
       <c r="D751" t="s">
         <v>753</v>
@@ -14944,7 +14944,7 @@
         <v>79</v>
       </c>
       <c r="C752">
-        <v>7100</v>
+        <v>7010</v>
       </c>
       <c r="D752" t="s">
         <v>754</v>
@@ -14958,7 +14958,7 @@
         <v>80</v>
       </c>
       <c r="C753">
-        <v>7100</v>
+        <v>7040</v>
       </c>
       <c r="D753" t="s">
         <v>755</v>
@@ -14972,7 +14972,7 @@
         <v>81</v>
       </c>
       <c r="C754">
-        <v>7100</v>
+        <v>7030</v>
       </c>
       <c r="D754" t="s">
         <v>756</v>
@@ -14986,7 +14986,7 @@
         <v>82</v>
       </c>
       <c r="C755">
-        <v>7100</v>
+        <v>6990</v>
       </c>
       <c r="D755" t="s">
         <v>757</v>
@@ -15000,7 +15000,7 @@
         <v>83</v>
       </c>
       <c r="C756">
-        <v>7080</v>
+        <v>6930</v>
       </c>
       <c r="D756" t="s">
         <v>758</v>
@@ -15014,7 +15014,7 @@
         <v>84</v>
       </c>
       <c r="C757">
-        <v>6980</v>
+        <v>6850</v>
       </c>
       <c r="D757" t="s">
         <v>759</v>
@@ -15028,7 +15028,7 @@
         <v>85</v>
       </c>
       <c r="C758">
-        <v>6820</v>
+        <v>6730</v>
       </c>
       <c r="D758" t="s">
         <v>760</v>
@@ -15042,7 +15042,7 @@
         <v>86</v>
       </c>
       <c r="C759">
-        <v>6650</v>
+        <v>6610</v>
       </c>
       <c r="D759" t="s">
         <v>761</v>
@@ -15056,7 +15056,7 @@
         <v>87</v>
       </c>
       <c r="C760">
-        <v>6540</v>
+        <v>6500</v>
       </c>
       <c r="D760" t="s">
         <v>762</v>
@@ -15070,7 +15070,7 @@
         <v>88</v>
       </c>
       <c r="C761">
-        <v>6450</v>
+        <v>6360</v>
       </c>
       <c r="D761" t="s">
         <v>763</v>
@@ -15084,7 +15084,7 @@
         <v>89</v>
       </c>
       <c r="C762">
-        <v>6330</v>
+        <v>6180</v>
       </c>
       <c r="D762" t="s">
         <v>764</v>
@@ -15098,7 +15098,7 @@
         <v>90</v>
       </c>
       <c r="C763">
-        <v>6220</v>
+        <v>6030</v>
       </c>
       <c r="D763" t="s">
         <v>765</v>
@@ -15112,7 +15112,7 @@
         <v>91</v>
       </c>
       <c r="C764">
-        <v>6040</v>
+        <v>5890</v>
       </c>
       <c r="D764" t="s">
         <v>766</v>
@@ -15126,7 +15126,7 @@
         <v>92</v>
       </c>
       <c r="C765">
-        <v>5920</v>
+        <v>5780</v>
       </c>
       <c r="D765" t="s">
         <v>767</v>
@@ -15140,7 +15140,7 @@
         <v>93</v>
       </c>
       <c r="C766">
-        <v>5830</v>
+        <v>5680</v>
       </c>
       <c r="D766" t="s">
         <v>768</v>
@@ -15154,7 +15154,7 @@
         <v>94</v>
       </c>
       <c r="C767">
-        <v>5670</v>
+        <v>5570</v>
       </c>
       <c r="D767" t="s">
         <v>769</v>
@@ -15168,7 +15168,7 @@
         <v>95</v>
       </c>
       <c r="C768">
-        <v>5580</v>
+        <v>5450</v>
       </c>
       <c r="D768" t="s">
         <v>770</v>
@@ -15182,7 +15182,7 @@
         <v>96</v>
       </c>
       <c r="C769">
-        <v>5470</v>
+        <v>5340</v>
       </c>
       <c r="D769" t="s">
         <v>771</v>
@@ -15196,7 +15196,7 @@
         <v>1</v>
       </c>
       <c r="C770">
-        <v>5460</v>
+        <v>5350</v>
       </c>
       <c r="D770" t="s">
         <v>772</v>
@@ -15210,7 +15210,7 @@
         <v>2</v>
       </c>
       <c r="C771">
-        <v>5420</v>
+        <v>5300</v>
       </c>
       <c r="D771" t="s">
         <v>773</v>
@@ -15224,7 +15224,7 @@
         <v>3</v>
       </c>
       <c r="C772">
-        <v>5360</v>
+        <v>5240</v>
       </c>
       <c r="D772" t="s">
         <v>774</v>
@@ -15238,7 +15238,7 @@
         <v>4</v>
       </c>
       <c r="C773">
-        <v>5280</v>
+        <v>5170</v>
       </c>
       <c r="D773" t="s">
         <v>775</v>
@@ -15252,7 +15252,7 @@
         <v>5</v>
       </c>
       <c r="C774">
-        <v>5220</v>
+        <v>5100</v>
       </c>
       <c r="D774" t="s">
         <v>776</v>
@@ -15266,7 +15266,7 @@
         <v>6</v>
       </c>
       <c r="C775">
-        <v>5180</v>
+        <v>5070</v>
       </c>
       <c r="D775" t="s">
         <v>777</v>
@@ -15280,7 +15280,7 @@
         <v>7</v>
       </c>
       <c r="C776">
-        <v>5160</v>
+        <v>5050</v>
       </c>
       <c r="D776" t="s">
         <v>778</v>
@@ -15294,7 +15294,7 @@
         <v>8</v>
       </c>
       <c r="C777">
-        <v>5140</v>
+        <v>5050</v>
       </c>
       <c r="D777" t="s">
         <v>779</v>
@@ -15308,7 +15308,7 @@
         <v>9</v>
       </c>
       <c r="C778">
-        <v>5120</v>
+        <v>5050</v>
       </c>
       <c r="D778" t="s">
         <v>780</v>
@@ -15322,7 +15322,7 @@
         <v>10</v>
       </c>
       <c r="C779">
-        <v>5100</v>
+        <v>5050</v>
       </c>
       <c r="D779" t="s">
         <v>781</v>
@@ -15336,7 +15336,7 @@
         <v>11</v>
       </c>
       <c r="C780">
-        <v>5100</v>
+        <v>5050</v>
       </c>
       <c r="D780" t="s">
         <v>782</v>
@@ -15350,7 +15350,7 @@
         <v>12</v>
       </c>
       <c r="C781">
-        <v>5120</v>
+        <v>5080</v>
       </c>
       <c r="D781" t="s">
         <v>783</v>
@@ -15364,7 +15364,7 @@
         <v>13</v>
       </c>
       <c r="C782">
-        <v>5120</v>
+        <v>5110</v>
       </c>
       <c r="D782" t="s">
         <v>784</v>
@@ -15378,7 +15378,7 @@
         <v>14</v>
       </c>
       <c r="C783">
-        <v>5140</v>
+        <v>5130</v>
       </c>
       <c r="D783" t="s">
         <v>785</v>
@@ -15420,7 +15420,7 @@
         <v>17</v>
       </c>
       <c r="C786">
-        <v>5180</v>
+        <v>5160</v>
       </c>
       <c r="D786" t="s">
         <v>788</v>
@@ -15434,7 +15434,7 @@
         <v>18</v>
       </c>
       <c r="C787">
-        <v>5190</v>
+        <v>5160</v>
       </c>
       <c r="D787" t="s">
         <v>789</v>
@@ -15448,7 +15448,7 @@
         <v>19</v>
       </c>
       <c r="C788">
-        <v>5210</v>
+        <v>5170</v>
       </c>
       <c r="D788" t="s">
         <v>790</v>
@@ -15462,7 +15462,7 @@
         <v>20</v>
       </c>
       <c r="C789">
-        <v>5250</v>
+        <v>5180</v>
       </c>
       <c r="D789" t="s">
         <v>791</v>
@@ -15476,7 +15476,7 @@
         <v>21</v>
       </c>
       <c r="C790">
-        <v>5290</v>
+        <v>5200</v>
       </c>
       <c r="D790" t="s">
         <v>792</v>
@@ -15490,7 +15490,7 @@
         <v>22</v>
       </c>
       <c r="C791">
-        <v>5360</v>
+        <v>5250</v>
       </c>
       <c r="D791" t="s">
         <v>793</v>
@@ -15504,7 +15504,7 @@
         <v>23</v>
       </c>
       <c r="C792">
-        <v>5450</v>
+        <v>5330</v>
       </c>
       <c r="D792" t="s">
         <v>794</v>
@@ -15518,7 +15518,7 @@
         <v>24</v>
       </c>
       <c r="C793">
-        <v>5560</v>
+        <v>5420</v>
       </c>
       <c r="D793" t="s">
         <v>795</v>
@@ -15532,7 +15532,7 @@
         <v>25</v>
       </c>
       <c r="C794">
-        <v>5690</v>
+        <v>5540</v>
       </c>
       <c r="D794" t="s">
         <v>796</v>
@@ -15546,7 +15546,7 @@
         <v>26</v>
       </c>
       <c r="C795">
-        <v>5830</v>
+        <v>5670</v>
       </c>
       <c r="D795" t="s">
         <v>797</v>
@@ -15560,7 +15560,7 @@
         <v>27</v>
       </c>
       <c r="C796">
-        <v>5980</v>
+        <v>5800</v>
       </c>
       <c r="D796" t="s">
         <v>798</v>
@@ -15574,7 +15574,7 @@
         <v>28</v>
       </c>
       <c r="C797">
-        <v>6140</v>
+        <v>5940</v>
       </c>
       <c r="D797" t="s">
         <v>799</v>
@@ -15588,7 +15588,7 @@
         <v>29</v>
       </c>
       <c r="C798">
-        <v>6290</v>
+        <v>6080</v>
       </c>
       <c r="D798" t="s">
         <v>800</v>
@@ -15602,7 +15602,7 @@
         <v>30</v>
       </c>
       <c r="C799">
-        <v>6420</v>
+        <v>6200</v>
       </c>
       <c r="D799" t="s">
         <v>801</v>
@@ -15616,7 +15616,7 @@
         <v>31</v>
       </c>
       <c r="C800">
-        <v>6530</v>
+        <v>6300</v>
       </c>
       <c r="D800" t="s">
         <v>802</v>
@@ -15630,7 +15630,7 @@
         <v>32</v>
       </c>
       <c r="C801">
-        <v>6610</v>
+        <v>6380</v>
       </c>
       <c r="D801" t="s">
         <v>803</v>
@@ -15644,7 +15644,7 @@
         <v>33</v>
       </c>
       <c r="C802">
-        <v>6650</v>
+        <v>6440</v>
       </c>
       <c r="D802" t="s">
         <v>804</v>
@@ -15658,7 +15658,7 @@
         <v>34</v>
       </c>
       <c r="C803">
-        <v>6650</v>
+        <v>6480</v>
       </c>
       <c r="D803" t="s">
         <v>805</v>
@@ -15672,7 +15672,7 @@
         <v>35</v>
       </c>
       <c r="C804">
-        <v>6650</v>
+        <v>6500</v>
       </c>
       <c r="D804" t="s">
         <v>806</v>
@@ -15686,7 +15686,7 @@
         <v>36</v>
       </c>
       <c r="C805">
-        <v>6630</v>
+        <v>6500</v>
       </c>
       <c r="D805" t="s">
         <v>807</v>
@@ -15700,7 +15700,7 @@
         <v>37</v>
       </c>
       <c r="C806">
-        <v>6560</v>
+        <v>6460</v>
       </c>
       <c r="D806" t="s">
         <v>808</v>
@@ -15714,7 +15714,7 @@
         <v>38</v>
       </c>
       <c r="C807">
-        <v>6490</v>
+        <v>6400</v>
       </c>
       <c r="D807" t="s">
         <v>809</v>
@@ -15728,7 +15728,7 @@
         <v>39</v>
       </c>
       <c r="C808">
-        <v>6400</v>
+        <v>6330</v>
       </c>
       <c r="D808" t="s">
         <v>810</v>
@@ -15742,7 +15742,7 @@
         <v>40</v>
       </c>
       <c r="C809">
-        <v>6310</v>
+        <v>6240</v>
       </c>
       <c r="D809" t="s">
         <v>811</v>
@@ -15756,7 +15756,7 @@
         <v>41</v>
       </c>
       <c r="C810">
-        <v>6220</v>
+        <v>6120</v>
       </c>
       <c r="D810" t="s">
         <v>812</v>
@@ -15770,7 +15770,7 @@
         <v>42</v>
       </c>
       <c r="C811">
-        <v>6130</v>
+        <v>6010</v>
       </c>
       <c r="D811" t="s">
         <v>813</v>
@@ -15784,7 +15784,7 @@
         <v>43</v>
       </c>
       <c r="C812">
-        <v>6050</v>
+        <v>5900</v>
       </c>
       <c r="D812" t="s">
         <v>814</v>
@@ -15798,7 +15798,7 @@
         <v>44</v>
       </c>
       <c r="C813">
-        <v>5980</v>
+        <v>5790</v>
       </c>
       <c r="D813" t="s">
         <v>815</v>
@@ -15812,7 +15812,7 @@
         <v>45</v>
       </c>
       <c r="C814">
-        <v>5910</v>
+        <v>5680</v>
       </c>
       <c r="D814" t="s">
         <v>816</v>
@@ -15826,7 +15826,7 @@
         <v>46</v>
       </c>
       <c r="C815">
-        <v>5860</v>
+        <v>5570</v>
       </c>
       <c r="D815" t="s">
         <v>817</v>
@@ -15840,7 +15840,7 @@
         <v>47</v>
       </c>
       <c r="C816">
-        <v>5800</v>
+        <v>5470</v>
       </c>
       <c r="D816" t="s">
         <v>818</v>
@@ -15854,7 +15854,7 @@
         <v>48</v>
       </c>
       <c r="C817">
-        <v>5750</v>
+        <v>5380</v>
       </c>
       <c r="D817" t="s">
         <v>819</v>
@@ -15868,7 +15868,7 @@
         <v>49</v>
       </c>
       <c r="C818">
-        <v>5710</v>
+        <v>5300</v>
       </c>
       <c r="D818" t="s">
         <v>820</v>
@@ -15882,7 +15882,7 @@
         <v>50</v>
       </c>
       <c r="C819">
-        <v>5670</v>
+        <v>5230</v>
       </c>
       <c r="D819" t="s">
         <v>821</v>
@@ -15896,7 +15896,7 @@
         <v>51</v>
       </c>
       <c r="C820">
-        <v>5640</v>
+        <v>5170</v>
       </c>
       <c r="D820" t="s">
         <v>822</v>
@@ -15910,7 +15910,7 @@
         <v>52</v>
       </c>
       <c r="C821">
-        <v>5620</v>
+        <v>5130</v>
       </c>
       <c r="D821" t="s">
         <v>823</v>
@@ -15924,7 +15924,7 @@
         <v>53</v>
       </c>
       <c r="C822">
-        <v>5600</v>
+        <v>5100</v>
       </c>
       <c r="D822" t="s">
         <v>824</v>
@@ -15938,7 +15938,7 @@
         <v>54</v>
       </c>
       <c r="C823">
-        <v>5600</v>
+        <v>5090</v>
       </c>
       <c r="D823" t="s">
         <v>825</v>
@@ -15952,7 +15952,7 @@
         <v>55</v>
       </c>
       <c r="C824">
-        <v>5600</v>
+        <v>5090</v>
       </c>
       <c r="D824" t="s">
         <v>826</v>
@@ -15966,7 +15966,7 @@
         <v>56</v>
       </c>
       <c r="C825">
-        <v>5600</v>
+        <v>5110</v>
       </c>
       <c r="D825" t="s">
         <v>827</v>
@@ -15980,7 +15980,7 @@
         <v>57</v>
       </c>
       <c r="C826">
-        <v>5610</v>
+        <v>5130</v>
       </c>
       <c r="D826" t="s">
         <v>828</v>
@@ -15994,7 +15994,7 @@
         <v>58</v>
       </c>
       <c r="C827">
-        <v>5620</v>
+        <v>5160</v>
       </c>
       <c r="D827" t="s">
         <v>829</v>
@@ -16008,7 +16008,7 @@
         <v>59</v>
       </c>
       <c r="C828">
-        <v>5630</v>
+        <v>5200</v>
       </c>
       <c r="D828" t="s">
         <v>830</v>
@@ -16022,7 +16022,7 @@
         <v>60</v>
       </c>
       <c r="C829">
-        <v>5650</v>
+        <v>5250</v>
       </c>
       <c r="D829" t="s">
         <v>831</v>
@@ -16036,7 +16036,7 @@
         <v>61</v>
       </c>
       <c r="C830">
-        <v>5660</v>
+        <v>5290</v>
       </c>
       <c r="D830" t="s">
         <v>832</v>
@@ -16050,7 +16050,7 @@
         <v>62</v>
       </c>
       <c r="C831">
-        <v>5680</v>
+        <v>5350</v>
       </c>
       <c r="D831" t="s">
         <v>833</v>
@@ -16064,7 +16064,7 @@
         <v>63</v>
       </c>
       <c r="C832">
-        <v>5710</v>
+        <v>5410</v>
       </c>
       <c r="D832" t="s">
         <v>834</v>
@@ -16078,7 +16078,7 @@
         <v>64</v>
       </c>
       <c r="C833">
-        <v>5760</v>
+        <v>5480</v>
       </c>
       <c r="D833" t="s">
         <v>835</v>
@@ -16092,7 +16092,7 @@
         <v>65</v>
       </c>
       <c r="C834">
-        <v>5810</v>
+        <v>5570</v>
       </c>
       <c r="D834" t="s">
         <v>836</v>
@@ -16106,7 +16106,7 @@
         <v>66</v>
       </c>
       <c r="C835">
-        <v>5880</v>
+        <v>5660</v>
       </c>
       <c r="D835" t="s">
         <v>837</v>
@@ -16120,7 +16120,7 @@
         <v>67</v>
       </c>
       <c r="C836">
-        <v>5950</v>
+        <v>5760</v>
       </c>
       <c r="D836" t="s">
         <v>838</v>
@@ -16134,7 +16134,7 @@
         <v>68</v>
       </c>
       <c r="C837">
-        <v>6040</v>
+        <v>5860</v>
       </c>
       <c r="D837" t="s">
         <v>839</v>
@@ -16148,7 +16148,7 @@
         <v>69</v>
       </c>
       <c r="C838">
-        <v>6130</v>
+        <v>5960</v>
       </c>
       <c r="D838" t="s">
         <v>840</v>
@@ -16162,7 +16162,7 @@
         <v>70</v>
       </c>
       <c r="C839">
-        <v>6220</v>
+        <v>6070</v>
       </c>
       <c r="D839" t="s">
         <v>841</v>
@@ -16176,7 +16176,7 @@
         <v>71</v>
       </c>
       <c r="C840">
-        <v>6310</v>
+        <v>6160</v>
       </c>
       <c r="D840" t="s">
         <v>842</v>
@@ -16190,7 +16190,7 @@
         <v>72</v>
       </c>
       <c r="C841">
-        <v>6400</v>
+        <v>6260</v>
       </c>
       <c r="D841" t="s">
         <v>843</v>
@@ -16204,7 +16204,7 @@
         <v>73</v>
       </c>
       <c r="C842">
-        <v>6490</v>
+        <v>6360</v>
       </c>
       <c r="D842" t="s">
         <v>844</v>
@@ -16218,7 +16218,7 @@
         <v>74</v>
       </c>
       <c r="C843">
-        <v>6590</v>
+        <v>6470</v>
       </c>
       <c r="D843" t="s">
         <v>845</v>
@@ -16232,7 +16232,7 @@
         <v>75</v>
       </c>
       <c r="C844">
-        <v>6710</v>
+        <v>6580</v>
       </c>
       <c r="D844" t="s">
         <v>846</v>
@@ -16246,7 +16246,7 @@
         <v>76</v>
       </c>
       <c r="C845">
-        <v>6830</v>
+        <v>6700</v>
       </c>
       <c r="D845" t="s">
         <v>847</v>
@@ -16260,7 +16260,7 @@
         <v>77</v>
       </c>
       <c r="C846">
-        <v>6950</v>
+        <v>6820</v>
       </c>
       <c r="D846" t="s">
         <v>848</v>
@@ -16274,7 +16274,7 @@
         <v>78</v>
       </c>
       <c r="C847">
-        <v>7050</v>
+        <v>6910</v>
       </c>
       <c r="D847" t="s">
         <v>849</v>
@@ -16288,7 +16288,7 @@
         <v>79</v>
       </c>
       <c r="C848">
-        <v>7100</v>
+        <v>6940</v>
       </c>
       <c r="D848" t="s">
         <v>850</v>
@@ -16302,7 +16302,7 @@
         <v>80</v>
       </c>
       <c r="C849">
-        <v>7100</v>
+        <v>6950</v>
       </c>
       <c r="D849" t="s">
         <v>851</v>
@@ -16316,7 +16316,7 @@
         <v>81</v>
       </c>
       <c r="C850">
-        <v>7100</v>
+        <v>6950</v>
       </c>
       <c r="D850" t="s">
         <v>852</v>
@@ -16330,7 +16330,7 @@
         <v>82</v>
       </c>
       <c r="C851">
-        <v>7100</v>
+        <v>6940</v>
       </c>
       <c r="D851" t="s">
         <v>853</v>
@@ -16344,7 +16344,7 @@
         <v>83</v>
       </c>
       <c r="C852">
-        <v>7080</v>
+        <v>6930</v>
       </c>
       <c r="D852" t="s">
         <v>854</v>
@@ -16358,7 +16358,7 @@
         <v>84</v>
       </c>
       <c r="C853">
-        <v>7000</v>
+        <v>6880</v>
       </c>
       <c r="D853" t="s">
         <v>855</v>
@@ -16372,7 +16372,7 @@
         <v>85</v>
       </c>
       <c r="C854">
-        <v>6860</v>
+        <v>6780</v>
       </c>
       <c r="D854" t="s">
         <v>856</v>
@@ -16386,7 +16386,7 @@
         <v>86</v>
       </c>
       <c r="C855">
-        <v>6690</v>
+        <v>6680</v>
       </c>
       <c r="D855" t="s">
         <v>857</v>
@@ -16400,7 +16400,7 @@
         <v>87</v>
       </c>
       <c r="C856">
-        <v>6600</v>
+        <v>6560</v>
       </c>
       <c r="D856" t="s">
         <v>858</v>
@@ -16414,7 +16414,7 @@
         <v>88</v>
       </c>
       <c r="C857">
-        <v>6500</v>
+        <v>6450</v>
       </c>
       <c r="D857" t="s">
         <v>859</v>
@@ -16428,7 +16428,7 @@
         <v>89</v>
       </c>
       <c r="C858">
-        <v>6360</v>
+        <v>6300</v>
       </c>
       <c r="D858" t="s">
         <v>860</v>
@@ -16442,7 +16442,7 @@
         <v>90</v>
       </c>
       <c r="C859">
-        <v>6230</v>
+        <v>6170</v>
       </c>
       <c r="D859" t="s">
         <v>861</v>
@@ -16456,7 +16456,7 @@
         <v>91</v>
       </c>
       <c r="C860">
-        <v>6060</v>
+        <v>6020</v>
       </c>
       <c r="D860" t="s">
         <v>862</v>
@@ -16470,7 +16470,7 @@
         <v>92</v>
       </c>
       <c r="C861">
-        <v>5950</v>
+        <v>5890</v>
       </c>
       <c r="D861" t="s">
         <v>863</v>
@@ -16484,7 +16484,7 @@
         <v>93</v>
       </c>
       <c r="C862">
-        <v>5870</v>
+        <v>5730</v>
       </c>
       <c r="D862" t="s">
         <v>864</v>
@@ -16498,7 +16498,7 @@
         <v>94</v>
       </c>
       <c r="C863">
-        <v>5720</v>
+        <v>5590</v>
       </c>
       <c r="D863" t="s">
         <v>865</v>
@@ -16512,7 +16512,7 @@
         <v>95</v>
       </c>
       <c r="C864">
-        <v>5630</v>
+        <v>5480</v>
       </c>
       <c r="D864" t="s">
         <v>866</v>
@@ -16526,7 +16526,7 @@
         <v>96</v>
       </c>
       <c r="C865">
-        <v>5520</v>
+        <v>5370</v>
       </c>
       <c r="D865" t="s">
         <v>867</v>
@@ -16540,7 +16540,7 @@
         <v>1</v>
       </c>
       <c r="C866">
-        <v>5180</v>
+        <v>5350</v>
       </c>
       <c r="D866" t="s">
         <v>868</v>
@@ -16554,7 +16554,7 @@
         <v>2</v>
       </c>
       <c r="C867">
-        <v>5160</v>
+        <v>5280</v>
       </c>
       <c r="D867" t="s">
         <v>869</v>
@@ -16568,7 +16568,7 @@
         <v>3</v>
       </c>
       <c r="C868">
-        <v>5150</v>
+        <v>5240</v>
       </c>
       <c r="D868" t="s">
         <v>870</v>
@@ -16582,7 +16582,7 @@
         <v>4</v>
       </c>
       <c r="C869">
-        <v>5140</v>
+        <v>5190</v>
       </c>
       <c r="D869" t="s">
         <v>871</v>
@@ -16596,7 +16596,7 @@
         <v>5</v>
       </c>
       <c r="C870">
-        <v>5120</v>
+        <v>5130</v>
       </c>
       <c r="D870" t="s">
         <v>872</v>
@@ -16610,7 +16610,7 @@
         <v>6</v>
       </c>
       <c r="C871">
-        <v>5110</v>
+        <v>5080</v>
       </c>
       <c r="D871" t="s">
         <v>873</v>
@@ -16624,7 +16624,7 @@
         <v>7</v>
       </c>
       <c r="C872">
-        <v>5100</v>
+        <v>5040</v>
       </c>
       <c r="D872" t="s">
         <v>874</v>
@@ -16638,7 +16638,7 @@
         <v>8</v>
       </c>
       <c r="C873">
-        <v>5080</v>
+        <v>5000</v>
       </c>
       <c r="D873" t="s">
         <v>875</v>
@@ -16652,7 +16652,7 @@
         <v>9</v>
       </c>
       <c r="C874">
-        <v>5070</v>
+        <v>4980</v>
       </c>
       <c r="D874" t="s">
         <v>876</v>
@@ -16666,7 +16666,7 @@
         <v>10</v>
       </c>
       <c r="C875">
-        <v>5060</v>
+        <v>4960</v>
       </c>
       <c r="D875" t="s">
         <v>877</v>
@@ -16680,7 +16680,7 @@
         <v>11</v>
       </c>
       <c r="C876">
-        <v>5060</v>
+        <v>4960</v>
       </c>
       <c r="D876" t="s">
         <v>878</v>
@@ -16694,7 +16694,7 @@
         <v>12</v>
       </c>
       <c r="C877">
-        <v>5050</v>
+        <v>4950</v>
       </c>
       <c r="D877" t="s">
         <v>879</v>
@@ -16708,7 +16708,7 @@
         <v>13</v>
       </c>
       <c r="C878">
-        <v>5050</v>
+        <v>4950</v>
       </c>
       <c r="D878" t="s">
         <v>880</v>
@@ -16722,7 +16722,7 @@
         <v>14</v>
       </c>
       <c r="C879">
-        <v>5050</v>
+        <v>4960</v>
       </c>
       <c r="D879" t="s">
         <v>881</v>
@@ -16736,7 +16736,7 @@
         <v>15</v>
       </c>
       <c r="C880">
-        <v>5060</v>
+        <v>4960</v>
       </c>
       <c r="D880" t="s">
         <v>882</v>
@@ -16750,7 +16750,7 @@
         <v>16</v>
       </c>
       <c r="C881">
-        <v>5070</v>
+        <v>4970</v>
       </c>
       <c r="D881" t="s">
         <v>883</v>
@@ -16764,7 +16764,7 @@
         <v>17</v>
       </c>
       <c r="C882">
-        <v>5090</v>
+        <v>4980</v>
       </c>
       <c r="D882" t="s">
         <v>884</v>
@@ -16778,7 +16778,7 @@
         <v>18</v>
       </c>
       <c r="C883">
-        <v>5100</v>
+        <v>5000</v>
       </c>
       <c r="D883" t="s">
         <v>885</v>
@@ -16792,7 +16792,7 @@
         <v>19</v>
       </c>
       <c r="C884">
-        <v>5120</v>
+        <v>5020</v>
       </c>
       <c r="D884" t="s">
         <v>886</v>
@@ -16806,7 +16806,7 @@
         <v>20</v>
       </c>
       <c r="C885">
-        <v>5130</v>
+        <v>5050</v>
       </c>
       <c r="D885" t="s">
         <v>887</v>
@@ -16820,7 +16820,7 @@
         <v>21</v>
       </c>
       <c r="C886">
-        <v>5140</v>
+        <v>5080</v>
       </c>
       <c r="D886" t="s">
         <v>888</v>
@@ -16834,7 +16834,7 @@
         <v>22</v>
       </c>
       <c r="C887">
-        <v>5150</v>
+        <v>5120</v>
       </c>
       <c r="D887" t="s">
         <v>889</v>
@@ -16848,7 +16848,7 @@
         <v>23</v>
       </c>
       <c r="C888">
-        <v>5150</v>
+        <v>5160</v>
       </c>
       <c r="D888" t="s">
         <v>890</v>
@@ -16862,7 +16862,7 @@
         <v>24</v>
       </c>
       <c r="C889">
-        <v>5160</v>
+        <v>5200</v>
       </c>
       <c r="D889" t="s">
         <v>891</v>
@@ -16876,7 +16876,7 @@
         <v>25</v>
       </c>
       <c r="C890">
-        <v>5170</v>
+        <v>5240</v>
       </c>
       <c r="D890" t="s">
         <v>892</v>
@@ -16890,7 +16890,7 @@
         <v>26</v>
       </c>
       <c r="C891">
-        <v>5190</v>
+        <v>5290</v>
       </c>
       <c r="D891" t="s">
         <v>893</v>
@@ -16904,7 +16904,7 @@
         <v>27</v>
       </c>
       <c r="C892">
-        <v>5220</v>
+        <v>5330</v>
       </c>
       <c r="D892" t="s">
         <v>894</v>
@@ -16918,7 +16918,7 @@
         <v>28</v>
       </c>
       <c r="C893">
-        <v>5250</v>
+        <v>5370</v>
       </c>
       <c r="D893" t="s">
         <v>895</v>
@@ -16932,7 +16932,7 @@
         <v>29</v>
       </c>
       <c r="C894">
-        <v>5280</v>
+        <v>5420</v>
       </c>
       <c r="D894" t="s">
         <v>896</v>
@@ -16946,7 +16946,7 @@
         <v>30</v>
       </c>
       <c r="C895">
-        <v>5310</v>
+        <v>5460</v>
       </c>
       <c r="D895" t="s">
         <v>897</v>
@@ -16960,7 +16960,7 @@
         <v>31</v>
       </c>
       <c r="C896">
-        <v>5330</v>
+        <v>5490</v>
       </c>
       <c r="D896" t="s">
         <v>898</v>
@@ -16974,7 +16974,7 @@
         <v>32</v>
       </c>
       <c r="C897">
-        <v>5350</v>
+        <v>5500</v>
       </c>
       <c r="D897" t="s">
         <v>899</v>
@@ -16988,7 +16988,7 @@
         <v>33</v>
       </c>
       <c r="C898">
-        <v>5350</v>
+        <v>5500</v>
       </c>
       <c r="D898" t="s">
         <v>900</v>
@@ -17002,7 +17002,7 @@
         <v>34</v>
       </c>
       <c r="C899">
-        <v>5320</v>
+        <v>5500</v>
       </c>
       <c r="D899" t="s">
         <v>901</v>
@@ -17016,7 +17016,7 @@
         <v>35</v>
       </c>
       <c r="C900">
-        <v>5280</v>
+        <v>5500</v>
       </c>
       <c r="D900" t="s">
         <v>902</v>
@@ -17030,7 +17030,7 @@
         <v>36</v>
       </c>
       <c r="C901">
-        <v>5210</v>
+        <v>5500</v>
       </c>
       <c r="D901" t="s">
         <v>903</v>
@@ -17044,7 +17044,7 @@
         <v>37</v>
       </c>
       <c r="C902">
-        <v>5110</v>
+        <v>5460</v>
       </c>
       <c r="D902" t="s">
         <v>904</v>
@@ -17058,7 +17058,7 @@
         <v>38</v>
       </c>
       <c r="C903">
-        <v>5000</v>
+        <v>5400</v>
       </c>
       <c r="D903" t="s">
         <v>905</v>
@@ -17072,7 +17072,7 @@
         <v>39</v>
       </c>
       <c r="C904">
-        <v>4870</v>
+        <v>5330</v>
       </c>
       <c r="D904" t="s">
         <v>906</v>
@@ -17086,7 +17086,7 @@
         <v>40</v>
       </c>
       <c r="C905">
-        <v>4730</v>
+        <v>5250</v>
       </c>
       <c r="D905" t="s">
         <v>907</v>
@@ -17100,7 +17100,7 @@
         <v>41</v>
       </c>
       <c r="C906">
-        <v>4590</v>
+        <v>5170</v>
       </c>
       <c r="D906" t="s">
         <v>908</v>
@@ -17114,7 +17114,7 @@
         <v>42</v>
       </c>
       <c r="C907">
-        <v>4460</v>
+        <v>5080</v>
       </c>
       <c r="D907" t="s">
         <v>909</v>
@@ -17128,7 +17128,7 @@
         <v>43</v>
       </c>
       <c r="C908">
-        <v>4330</v>
+        <v>5000</v>
       </c>
       <c r="D908" t="s">
         <v>910</v>
@@ -17142,7 +17142,7 @@
         <v>44</v>
       </c>
       <c r="C909">
-        <v>4220</v>
+        <v>4920</v>
       </c>
       <c r="D909" t="s">
         <v>911</v>
@@ -17156,7 +17156,7 @@
         <v>45</v>
       </c>
       <c r="C910">
-        <v>4120</v>
+        <v>4860</v>
       </c>
       <c r="D910" t="s">
         <v>912</v>
@@ -17170,7 +17170,7 @@
         <v>46</v>
       </c>
       <c r="C911">
-        <v>4050</v>
+        <v>4800</v>
       </c>
       <c r="D911" t="s">
         <v>913</v>
@@ -17184,7 +17184,7 @@
         <v>47</v>
       </c>
       <c r="C912">
-        <v>3980</v>
+        <v>4740</v>
       </c>
       <c r="D912" t="s">
         <v>914</v>
@@ -17198,7 +17198,7 @@
         <v>48</v>
       </c>
       <c r="C913">
-        <v>3940</v>
+        <v>4700</v>
       </c>
       <c r="D913" t="s">
         <v>915</v>
@@ -17212,7 +17212,7 @@
         <v>49</v>
       </c>
       <c r="C914">
-        <v>3910</v>
+        <v>4660</v>
       </c>
       <c r="D914" t="s">
         <v>916</v>
@@ -17226,7 +17226,7 @@
         <v>50</v>
       </c>
       <c r="C915">
-        <v>3890</v>
+        <v>4630</v>
       </c>
       <c r="D915" t="s">
         <v>917</v>
@@ -17240,7 +17240,7 @@
         <v>51</v>
       </c>
       <c r="C916">
-        <v>3870</v>
+        <v>4600</v>
       </c>
       <c r="D916" t="s">
         <v>918</v>
@@ -17254,7 +17254,7 @@
         <v>52</v>
       </c>
       <c r="C917">
-        <v>3870</v>
+        <v>4570</v>
       </c>
       <c r="D917" t="s">
         <v>919</v>
@@ -17268,7 +17268,7 @@
         <v>53</v>
       </c>
       <c r="C918">
-        <v>3870</v>
+        <v>4560</v>
       </c>
       <c r="D918" t="s">
         <v>920</v>
@@ -17282,7 +17282,7 @@
         <v>54</v>
       </c>
       <c r="C919">
-        <v>3880</v>
+        <v>4550</v>
       </c>
       <c r="D919" t="s">
         <v>921</v>
@@ -17296,7 +17296,7 @@
         <v>55</v>
       </c>
       <c r="C920">
-        <v>3900</v>
+        <v>4560</v>
       </c>
       <c r="D920" t="s">
         <v>922</v>
@@ -17310,7 +17310,7 @@
         <v>56</v>
       </c>
       <c r="C921">
-        <v>3920</v>
+        <v>4580</v>
       </c>
       <c r="D921" t="s">
         <v>923</v>
@@ -17324,7 +17324,7 @@
         <v>57</v>
       </c>
       <c r="C922">
-        <v>3960</v>
+        <v>4600</v>
       </c>
       <c r="D922" t="s">
         <v>924</v>
@@ -17338,7 +17338,7 @@
         <v>58</v>
       </c>
       <c r="C923">
-        <v>3990</v>
+        <v>4640</v>
       </c>
       <c r="D923" t="s">
         <v>925</v>
@@ -17352,7 +17352,7 @@
         <v>59</v>
       </c>
       <c r="C924">
-        <v>4040</v>
+        <v>4680</v>
       </c>
       <c r="D924" t="s">
         <v>926</v>
@@ -17366,7 +17366,7 @@
         <v>60</v>
       </c>
       <c r="C925">
-        <v>4090</v>
+        <v>4730</v>
       </c>
       <c r="D925" t="s">
         <v>927</v>
@@ -17380,7 +17380,7 @@
         <v>61</v>
       </c>
       <c r="C926">
-        <v>4160</v>
+        <v>4780</v>
       </c>
       <c r="D926" t="s">
         <v>928</v>
@@ -17394,7 +17394,7 @@
         <v>62</v>
       </c>
       <c r="C927">
-        <v>4230</v>
+        <v>4830</v>
       </c>
       <c r="D927" t="s">
         <v>929</v>
@@ -17408,7 +17408,7 @@
         <v>63</v>
       </c>
       <c r="C928">
-        <v>4310</v>
+        <v>4890</v>
       </c>
       <c r="D928" t="s">
         <v>930</v>
@@ -17422,7 +17422,7 @@
         <v>64</v>
       </c>
       <c r="C929">
-        <v>4410</v>
+        <v>4950</v>
       </c>
       <c r="D929" t="s">
         <v>931</v>
@@ -17436,7 +17436,7 @@
         <v>65</v>
       </c>
       <c r="C930">
-        <v>4510</v>
+        <v>5020</v>
       </c>
       <c r="D930" t="s">
         <v>932</v>
@@ -17450,7 +17450,7 @@
         <v>66</v>
       </c>
       <c r="C931">
-        <v>4630</v>
+        <v>5110</v>
       </c>
       <c r="D931" t="s">
         <v>933</v>
@@ -17464,7 +17464,7 @@
         <v>67</v>
       </c>
       <c r="C932">
-        <v>4760</v>
+        <v>5200</v>
       </c>
       <c r="D932" t="s">
         <v>934</v>
@@ -17478,7 +17478,7 @@
         <v>68</v>
       </c>
       <c r="C933">
-        <v>4900</v>
+        <v>5310</v>
       </c>
       <c r="D933" t="s">
         <v>935</v>
@@ -17492,7 +17492,7 @@
         <v>69</v>
       </c>
       <c r="C934">
-        <v>5050</v>
+        <v>5430</v>
       </c>
       <c r="D934" t="s">
         <v>936</v>
@@ -17506,7 +17506,7 @@
         <v>70</v>
       </c>
       <c r="C935">
-        <v>5200</v>
+        <v>5560</v>
       </c>
       <c r="D935" t="s">
         <v>937</v>
@@ -17520,7 +17520,7 @@
         <v>71</v>
       </c>
       <c r="C936">
-        <v>5340</v>
+        <v>5680</v>
       </c>
       <c r="D936" t="s">
         <v>938</v>
@@ -17534,7 +17534,7 @@
         <v>72</v>
       </c>
       <c r="C937">
-        <v>5490</v>
+        <v>5800</v>
       </c>
       <c r="D937" t="s">
         <v>939</v>
@@ -17548,7 +17548,7 @@
         <v>73</v>
       </c>
       <c r="C938">
-        <v>5630</v>
+        <v>5930</v>
       </c>
       <c r="D938" t="s">
         <v>940</v>
@@ -17562,7 +17562,7 @@
         <v>74</v>
       </c>
       <c r="C939">
-        <v>5770</v>
+        <v>6050</v>
       </c>
       <c r="D939" t="s">
         <v>941</v>
@@ -17576,7 +17576,7 @@
         <v>75</v>
       </c>
       <c r="C940">
-        <v>5910</v>
+        <v>6170</v>
       </c>
       <c r="D940" t="s">
         <v>942</v>
@@ -17590,7 +17590,7 @@
         <v>76</v>
       </c>
       <c r="C941">
-        <v>6050</v>
+        <v>6300</v>
       </c>
       <c r="D941" t="s">
         <v>943</v>
@@ -17604,7 +17604,7 @@
         <v>77</v>
       </c>
       <c r="C942">
-        <v>6180</v>
+        <v>6410</v>
       </c>
       <c r="D942" t="s">
         <v>944</v>
@@ -17618,7 +17618,7 @@
         <v>78</v>
       </c>
       <c r="C943">
-        <v>6300</v>
+        <v>6510</v>
       </c>
       <c r="D943" t="s">
         <v>945</v>
@@ -17632,7 +17632,7 @@
         <v>79</v>
       </c>
       <c r="C944">
-        <v>6400</v>
+        <v>6550</v>
       </c>
       <c r="D944" t="s">
         <v>946</v>
@@ -17646,7 +17646,7 @@
         <v>80</v>
       </c>
       <c r="C945">
-        <v>6470</v>
+        <v>6550</v>
       </c>
       <c r="D945" t="s">
         <v>947</v>
@@ -17660,7 +17660,7 @@
         <v>81</v>
       </c>
       <c r="C946">
-        <v>6520</v>
+        <v>6550</v>
       </c>
       <c r="D946" t="s">
         <v>948</v>
@@ -17674,7 +17674,7 @@
         <v>82</v>
       </c>
       <c r="C947">
-        <v>6530</v>
+        <v>6550</v>
       </c>
       <c r="D947" t="s">
         <v>949</v>
@@ -17688,7 +17688,7 @@
         <v>83</v>
       </c>
       <c r="C948">
-        <v>6490</v>
+        <v>6540</v>
       </c>
       <c r="D948" t="s">
         <v>950</v>
@@ -17702,7 +17702,7 @@
         <v>84</v>
       </c>
       <c r="C949">
-        <v>6410</v>
+        <v>6490</v>
       </c>
       <c r="D949" t="s">
         <v>951</v>
@@ -17716,7 +17716,7 @@
         <v>85</v>
       </c>
       <c r="C950">
-        <v>6260</v>
+        <v>6400</v>
       </c>
       <c r="D950" t="s">
         <v>952</v>
@@ -17730,7 +17730,7 @@
         <v>86</v>
       </c>
       <c r="C951">
-        <v>6090</v>
+        <v>6280</v>
       </c>
       <c r="D951" t="s">
         <v>953</v>
@@ -17744,7 +17744,7 @@
         <v>87</v>
       </c>
       <c r="C952">
-        <v>6000</v>
+        <v>6220</v>
       </c>
       <c r="D952" t="s">
         <v>954</v>
@@ -17758,7 +17758,7 @@
         <v>88</v>
       </c>
       <c r="C953">
-        <v>5910</v>
+        <v>6140</v>
       </c>
       <c r="D953" t="s">
         <v>955</v>
@@ -17772,7 +17772,7 @@
         <v>89</v>
       </c>
       <c r="C954">
-        <v>5790</v>
+        <v>6010</v>
       </c>
       <c r="D954" t="s">
         <v>956</v>
@@ -17786,7 +17786,7 @@
         <v>90</v>
       </c>
       <c r="C955">
-        <v>5690</v>
+        <v>5920</v>
       </c>
       <c r="D955" t="s">
         <v>957</v>
@@ -17800,7 +17800,7 @@
         <v>91</v>
       </c>
       <c r="C956">
-        <v>5510</v>
+        <v>5780</v>
       </c>
       <c r="D956" t="s">
         <v>958</v>
@@ -17814,7 +17814,7 @@
         <v>92</v>
       </c>
       <c r="C957">
-        <v>5400</v>
+        <v>5650</v>
       </c>
       <c r="D957" t="s">
         <v>959</v>
@@ -17828,7 +17828,7 @@
         <v>93</v>
       </c>
       <c r="C958">
-        <v>5320</v>
+        <v>5510</v>
       </c>
       <c r="D958" t="s">
         <v>960</v>
@@ -17842,7 +17842,7 @@
         <v>94</v>
       </c>
       <c r="C959">
-        <v>5170</v>
+        <v>5380</v>
       </c>
       <c r="D959" t="s">
         <v>961</v>
@@ -17856,7 +17856,7 @@
         <v>95</v>
       </c>
       <c r="C960">
-        <v>5150</v>
+        <v>5270</v>
       </c>
       <c r="D960" t="s">
         <v>962</v>
@@ -17870,7 +17870,7 @@
         <v>96</v>
       </c>
       <c r="C961">
-        <v>5120</v>
+        <v>5170</v>
       </c>
       <c r="D961" t="s">
         <v>963</v>

</xml_diff>